<commit_message>
Explicando melhor o projeto e interpretação no readme, adicionando imagens ao readme
</commit_message>
<xml_diff>
--- a/data/outputs/scenario_summary.xlsx
+++ b/data/outputs/scenario_summary.xlsx
@@ -426,7 +426,7 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>689268.9818224323</v>
+        <v>672842.7199907185</v>
       </c>
       <c r="C2">
         <v>0.005817047883905853</v>
@@ -446,7 +446,7 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>753598.7619498045</v>
+        <v>735646.9369003867</v>
       </c>
       <c r="C3">
         <v>0.005974087909148729</v>
@@ -466,13 +466,13 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>823330.0503195543</v>
+        <v>803722.3715759255</v>
       </c>
       <c r="C4">
         <v>0.006176066738024838</v>
       </c>
       <c r="D4">
-        <v>0.7592898349607641</v>
+        <v>0.7592898349607642</v>
       </c>
       <c r="E4">
         <v>14082.48227684434</v>

</xml_diff>

<commit_message>
correção staging e melhoria ecl
</commit_message>
<xml_diff>
--- a/data/outputs/scenario_summary.xlsx
+++ b/data/outputs/scenario_summary.xlsx
@@ -14,11 +14,41 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>scenario</t>
   </si>
   <si>
+    <t>input_weight</t>
+  </si>
+  <si>
+    <t>pd_multiplier</t>
+  </si>
+  <si>
+    <t>lgd_multiplier</t>
+  </si>
+  <si>
+    <t>unemployment_shift</t>
+  </si>
+  <si>
+    <t>selic_shift</t>
+  </si>
+  <si>
+    <t>gdp_shift</t>
+  </si>
+  <si>
+    <t>input_weight_sum</t>
+  </si>
+  <si>
+    <t>normalized_weight</t>
+  </si>
+  <si>
+    <t>weights_normalized</t>
+  </si>
+  <si>
+    <t>macro_reference_date</t>
+  </si>
+  <si>
     <t>total_ecl</t>
   </si>
   <si>
@@ -31,6 +61,15 @@
     <t>avg_ead</t>
   </si>
   <si>
+    <t>stage1_share</t>
+  </si>
+  <si>
+    <t>stage2_share</t>
+  </si>
+  <si>
+    <t>stage3_share</t>
+  </si>
+  <si>
     <t>stage2_plus_share</t>
   </si>
   <si>
@@ -41,6 +80,9 @@
   </si>
   <si>
     <t>severe</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
   </si>
 </sst>
 </file>
@@ -398,10 +440,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -420,65 +462,221 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="B2">
-        <v>428485.0218909638</v>
+        <v>0.6</v>
       </c>
       <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0.9999999999999999</v>
+      </c>
+      <c r="I2">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2">
+        <v>411574.9407520655</v>
+      </c>
+      <c r="M2">
         <v>0.003799504702758448</v>
       </c>
-      <c r="D2">
+      <c r="N2">
         <v>0.6898099741546282</v>
       </c>
-      <c r="E2">
+      <c r="O2">
         <v>14080.28925828435</v>
       </c>
-      <c r="F2">
-        <v>0.242125</v>
+      <c r="P2">
+        <v>0.765375</v>
+      </c>
+      <c r="Q2">
+        <v>0.180125</v>
+      </c>
+      <c r="R2">
+        <v>0.0545</v>
+      </c>
+      <c r="S2">
+        <v>0.234625</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B3">
-        <v>553174.2305278705</v>
+        <v>0.3</v>
       </c>
       <c r="C3">
+        <v>1.2</v>
+      </c>
+      <c r="D3">
+        <v>1.05</v>
+      </c>
+      <c r="E3">
+        <v>0.02</v>
+      </c>
+      <c r="F3">
+        <v>0.02</v>
+      </c>
+      <c r="G3">
+        <v>-0.02</v>
+      </c>
+      <c r="H3">
+        <v>0.9999999999999999</v>
+      </c>
+      <c r="I3">
+        <v>0.3</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
+      <c r="K3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3">
+        <v>517481.4750927588</v>
+      </c>
+      <c r="M3">
         <v>0.004559405643310138</v>
       </c>
-      <c r="D3">
+      <c r="N3">
         <v>0.7243004728623595</v>
       </c>
-      <c r="E3">
+      <c r="O3">
         <v>14080.28925828435</v>
       </c>
-      <c r="F3">
-        <v>0.268625</v>
+      <c r="P3">
+        <v>0.765375</v>
+      </c>
+      <c r="Q3">
+        <v>0.180125</v>
+      </c>
+      <c r="R3">
+        <v>0.0545</v>
+      </c>
+      <c r="S3">
+        <v>0.234625</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="B4">
-        <v>722138.7300881529</v>
+        <v>0.1</v>
       </c>
       <c r="C4">
+        <v>1.45</v>
+      </c>
+      <c r="D4">
+        <v>1.1</v>
+      </c>
+      <c r="E4">
+        <v>0.04</v>
+      </c>
+      <c r="F4">
+        <v>0.04</v>
+      </c>
+      <c r="G4">
+        <v>-0.04</v>
+      </c>
+      <c r="H4">
+        <v>0.9999999999999999</v>
+      </c>
+      <c r="I4">
+        <v>0.1</v>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
+      <c r="K4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4">
+        <v>652983.3625199589</v>
+      </c>
+      <c r="M4">
         <v>0.00550928181899975</v>
       </c>
-      <c r="D4">
+      <c r="N4">
         <v>0.758665212049864</v>
       </c>
-      <c r="E4">
+      <c r="O4">
         <v>14080.28925828435</v>
       </c>
-      <c r="F4">
-        <v>0.3115</v>
+      <c r="P4">
+        <v>0.765375</v>
+      </c>
+      <c r="Q4">
+        <v>0.180125</v>
+      </c>
+      <c r="R4">
+        <v>0.0545</v>
+      </c>
+      <c r="S4">
+        <v>0.234625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>